<commit_message>
last push, i hope (adj literature)
</commit_message>
<xml_diff>
--- a/literatur_dan_data/data_mentah/template_data.xlsx
+++ b/literatur_dan_data/data_mentah/template_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kuliah\Sem 6\VisualData\UAS_VD\literatur_dan_data\data_mentah\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAC221C-718D-4A61-99F3-2AB0C6FAD229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9B4B45-F82E-4F95-8E0A-C014208A5D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="METADATA_SOURCES" sheetId="2" r:id="rId1"/>
@@ -1972,9 +1972,6 @@
     <t>Penandaan sendiri</t>
   </si>
   <si>
-    <t>DIISI = arus antarprovinsi; EXCLUDE_DIAGONAL = sel asal=tujuan</t>
-  </si>
-  <si>
     <t>Kode rujukan ke sheet METADATA_SOURCES</t>
   </si>
   <si>
@@ -2192,6 +2189,9 @@
   </si>
   <si>
     <t>status_observasi</t>
+  </si>
+  <si>
+    <t>isi = arus antarprovinsi; keluar = sel asalsama dengan tujuan</t>
   </si>
 </sst>
 </file>
@@ -2408,7 +2408,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2501,6 +2501,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2511,17 +2514,31 @@
   </cellStyles>
   <dxfs count="88">
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -2538,11 +2555,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -2556,7 +2569,7 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
       <border diagonalUp="0" diagonalDown="0">
@@ -2569,18 +2582,20 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -2594,10 +2609,9 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -2608,58 +2622,20 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -2673,71 +2649,9 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -2751,38 +2665,33 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
+        <vertical style="thin">
           <color indexed="64"/>
-        </bottom>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
+        <color theme="1"/>
         <name val="Calibri"/>
-        <scheme val="none"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -2790,8 +2699,12 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top/>
-        <bottom/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
         <vertical style="thin">
           <color indexed="64"/>
         </vertical>
@@ -2799,6 +2712,194 @@
           <color indexed="64"/>
         </horizontal>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -3013,6 +3114,13 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -3022,13 +3130,6 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -4180,340 +4281,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -4957,6 +4724,296 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4971,55 +5028,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{05A74CF1-03A1-407E-8377-AE50F1676D81}" name="Table8" displayName="Table8" ref="A1:I12" totalsRowShown="0" headerRowDxfId="87" headerRowBorderDxfId="86" tableBorderDxfId="85" totalsRowBorderDxfId="84">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{05A74CF1-03A1-407E-8377-AE50F1676D81}" name="Table8" displayName="Table8" ref="A1:I12" totalsRowShown="0" headerRowDxfId="77" headerRowBorderDxfId="76" tableBorderDxfId="75" totalsRowBorderDxfId="74">
   <autoFilter ref="A1:I12" xr:uid="{05A74CF1-03A1-407E-8377-AE50F1676D81}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{FBA84A87-B07A-4C56-BD0D-73789F0D1486}" name="ID_Sumber" dataDxfId="83"/>
-    <tableColumn id="2" xr3:uid="{ED058142-2F40-4B04-9813-E9C660D3E5CF}" name="Topik/Sheet" dataDxfId="82"/>
-    <tableColumn id="3" xr3:uid="{FA43377D-AB27-424C-AAC7-F7A73B6C94BD}" name="Judul Tabel/Publikasi" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{F7D61127-9A81-4F15-BB79-25F92035BB09}" name="Instansi" dataDxfId="80"/>
-    <tableColumn id="5" xr3:uid="{EF861922-D9CE-47F1-9B96-2118F64C2F22}" name="Periode" dataDxfId="79"/>
-    <tableColumn id="6" xr3:uid="{8FBF2AEA-983F-4E16-B25E-3BF5547A783F}" name="URL" dataDxfId="78" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{2500CAA4-CD0E-4AA5-AAF2-0B68C6F25079}" name="Tanggal_Akses" dataDxfId="77"/>
-    <tableColumn id="8" xr3:uid="{A47D88EF-3CE3-4587-8513-46D3CEAEAFAE}" name="Lampiran/Halaman" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{B81325CA-194D-4837-9E15-B7FB06816AB1}" name="Definisi/Catatan" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{FBA84A87-B07A-4C56-BD0D-73789F0D1486}" name="ID_Sumber" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{ED058142-2F40-4B04-9813-E9C660D3E5CF}" name="Topik/Sheet" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{FA43377D-AB27-424C-AAC7-F7A73B6C94BD}" name="Judul Tabel/Publikasi" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{F7D61127-9A81-4F15-BB79-25F92035BB09}" name="Instansi" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{EF861922-D9CE-47F1-9B96-2118F64C2F22}" name="Periode" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{8FBF2AEA-983F-4E16-B25E-3BF5547A783F}" name="URL" dataDxfId="68" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{2500CAA4-CD0E-4AA5-AAF2-0B68C6F25079}" name="Tanggal_Akses" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{A47D88EF-3CE3-4587-8513-46D3CEAEAFAE}" name="Lampiran/Halaman" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{B81325CA-194D-4837-9E15-B7FB06816AB1}" name="Definisi/Catatan" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0C36B66F-E5C7-40B0-9436-C40F978E5109}" name="Table7" displayName="Table7" ref="A1:H49" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71" totalsRowBorderDxfId="70">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0C36B66F-E5C7-40B0-9436-C40F978E5109}" name="Table7" displayName="Table7" ref="A1:H49" totalsRowShown="0" headerRowDxfId="64" dataDxfId="62" headerRowBorderDxfId="63" tableBorderDxfId="61" totalsRowBorderDxfId="60">
   <autoFilter ref="A1:H49" xr:uid="{0C36B66F-E5C7-40B0-9436-C40F978E5109}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C3BD0185-D545-45E4-BD34-00278A104878}" name="Sheet" dataDxfId="69"/>
-    <tableColumn id="2" xr3:uid="{C55E2377-6D13-4384-95FA-B54EA53DA878}" name="Nama_Variabel" dataDxfId="68"/>
-    <tableColumn id="3" xr3:uid="{A6CBB1D6-6484-45D9-8492-488F8C91F310}" name="Definisi" dataDxfId="67"/>
-    <tableColumn id="4" xr3:uid="{090F08DA-7B1C-40B8-A19E-CFEC7717B4F0}" name="Satuan" dataDxfId="66"/>
-    <tableColumn id="5" xr3:uid="{3846AE14-72E6-4AB1-A8A0-8D13B89C649B}" name="Tipe_Data" dataDxfId="65"/>
-    <tableColumn id="6" xr3:uid="{2FEBD57C-793A-47A0-B790-F613CB1CE07E}" name="Periode" dataDxfId="64"/>
-    <tableColumn id="7" xr3:uid="{696C2E29-1042-48E5-81BD-3776A68CCBDC}" name="Sumber" dataDxfId="63"/>
-    <tableColumn id="8" xr3:uid="{DCABD5BA-160F-4D70-8F16-7CBCF47A1342}" name="Transformasi/Rumus" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{C3BD0185-D545-45E4-BD34-00278A104878}" name="Sheet" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{C55E2377-6D13-4384-95FA-B54EA53DA878}" name="Nama_Variabel" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{A6CBB1D6-6484-45D9-8492-488F8C91F310}" name="Definisi" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{090F08DA-7B1C-40B8-A19E-CFEC7717B4F0}" name="Satuan" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{3846AE14-72E6-4AB1-A8A0-8D13B89C649B}" name="Tipe_Data" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{2FEBD57C-793A-47A0-B790-F613CB1CE07E}" name="Periode" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{696C2E29-1042-48E5-81BD-3776A68CCBDC}" name="Sumber" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{DCABD5BA-160F-4D70-8F16-7CBCF47A1342}" name="Transformasi/Rumus" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblFLOWOD" displayName="tblFLOWOD" ref="A1:I1157" dataDxfId="61" totalsRowDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblFLOWOD" displayName="tblFLOWOD" ref="A1:I1157" dataDxfId="10" totalsRowDxfId="9">
   <autoFilter ref="A1:I1157" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="kode_asal" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="nama_asal" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="kode_tujuan" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="nama_tujuan" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="jumlah_migran" dataDxfId="55"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="jenis_migrasi" dataDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="tahun_data" dataDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status_observasi" dataDxfId="52">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="kode_asal" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="nama_asal" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="kode_tujuan" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="nama_tujuan" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="jumlah_migran" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="jenis_migrasi" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="tahun_data" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status_observasi" dataDxfId="1">
       <calculatedColumnFormula>IF(tblFLOWOD[[#This Row],[nama_asal]]=tblFLOWOD[[#This Row],[nama_tujuan]],"keluar","isi")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="id_sumber" dataDxfId="51">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="id_sumber" dataDxfId="0">
       <calculatedColumnFormula>METADATA_SOURCES!$A$2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5028,20 +5085,20 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblMultivariat" displayName="tblMultivariat" ref="A1:K35" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblMultivariat" displayName="tblMultivariat" ref="A1:K35" dataDxfId="51">
   <autoFilter ref="A1:K35" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="kode_provinsi" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="nama_provinsi" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="ipm" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="uhh" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="hls" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="rls" dataDxfId="44"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="pengeluaran_per_kapita" dataDxfId="43"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="persentase_miskin" dataDxfId="42"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="tpt" dataDxfId="41"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="kepadatan_penduduk" dataDxfId="40"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="id_sumber" dataDxfId="39">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="kode_provinsi" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="nama_provinsi" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="ipm" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="uhh" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="hls" dataDxfId="46"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="rls" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="pengeluaran_per_kapita" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="persentase_miskin" dataDxfId="43"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="tpt" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="kepadatan_penduduk" dataDxfId="41"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="id_sumber" dataDxfId="40">
       <calculatedColumnFormula>CONCATENATE(METADATA_SOURCES!$A$3,"; ",METADATA_SOURCES!$A$4)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5050,24 +5107,24 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblGeo" displayName="tblGeo" ref="A1:J515" dataDxfId="38" totalsRowDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblGeo" displayName="tblGeo" ref="A1:J515" dataDxfId="39" totalsRowDxfId="38">
   <autoFilter ref="A1:J515" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J515">
     <sortCondition ref="A2:A515"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="kode_bps" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="nama_kabkota" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="kode_provinsi" dataDxfId="34">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="kode_bps" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="nama_kabkota" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="kode_provinsi" dataDxfId="35">
       <calculatedColumnFormula>LEFT(A2,2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="nama_provinsi" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="persentase_miskin" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="ipm" dataDxfId="31"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="pdrb_per_kapita" dataDxfId="30"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="tpt" dataDxfId="29"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="jumlah_penduduk" dataDxfId="28"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0200-000011000000}" name="id_sumber" dataDxfId="27">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="nama_provinsi" dataDxfId="34"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="persentase_miskin" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="ipm" dataDxfId="32"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="pdrb_per_kapita" dataDxfId="31"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="tpt" dataDxfId="30"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="jumlah_penduduk" dataDxfId="29"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0200-000011000000}" name="id_sumber" dataDxfId="28">
       <calculatedColumnFormula>CONCATENATE(METADATA_SOURCES!$A$5,"; ",METADATA_SOURCES!$A$6,"; ",METADATA_SOURCES!$A$7,"; ",METADATA_SOURCES!$A$8,"; ",METADATA_SOURCES!$A$9,"; ",METADATA_SOURCES!$A$10,"; ",METADATA_SOURCES!$A$11)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5076,15 +5133,15 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C9804DE7-B41C-43BA-931C-E29714FFAF6B}" name="Table4" displayName="Table4" ref="A1:F143" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C9804DE7-B41C-43BA-931C-E29714FFAF6B}" name="Table4" displayName="Table4" ref="A1:F143" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:F143" xr:uid="{C9804DE7-B41C-43BA-931C-E29714FFAF6B}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{CA32B770-B1D3-4DFD-A276-C72ACB437E3D}" name="kode_asal" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{CD4B4A66-1DB5-4464-B7A6-94B5D9FF0A0C}" name="nama_asal" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{609E1D10-3D37-4E5E-85D1-DD7F9EBCEBD9}" name="kode_tujuan" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{56F532E0-FDD1-48C6-84AD-1170C48E37BA}" name="nama_tujuan" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{D3A6D151-99D6-4B9E-AEBE-9C4B93229A56}" name="jumlah_komuter" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{18042B5F-29D8-4319-AC1C-CE39FD6DA62B}" name="id_sumber" dataDxfId="19">
+    <tableColumn id="1" xr3:uid="{CA32B770-B1D3-4DFD-A276-C72ACB437E3D}" name="kode_asal" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{CD4B4A66-1DB5-4464-B7A6-94B5D9FF0A0C}" name="nama_asal" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{609E1D10-3D37-4E5E-85D1-DD7F9EBCEBD9}" name="kode_tujuan" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{56F532E0-FDD1-48C6-84AD-1170C48E37BA}" name="nama_tujuan" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{D3A6D151-99D6-4B9E-AEBE-9C4B93229A56}" name="jumlah_komuter" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{18042B5F-29D8-4319-AC1C-CE39FD6DA62B}" name="id_sumber" dataDxfId="20">
       <calculatedColumnFormula>METADATA_SOURCES!$A$12</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5093,29 +5150,29 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{3344DD33-6A3C-4F09-9581-C7EB980F886F}" name="Table5" displayName="Table5" ref="A1:E67" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{3344DD33-6A3C-4F09-9581-C7EB980F886F}" name="Table5" displayName="Table5" ref="A1:E67" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="17" tableBorderDxfId="18" totalsRowBorderDxfId="16">
   <autoFilter ref="A1:E67" xr:uid="{3344DD33-6A3C-4F09-9581-C7EB980F886F}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A97C526F-F4CF-439B-94B7-1ACC3B0D52B8}" name="kode_asal" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{A06EB03B-EFA2-428E-8750-2625B01CC79E}" name="nama_asal" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{915F2F13-451B-4692-85C8-931B037F0D1D}" name="kode_tujuan" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{CA49676B-7235-4E1F-80E5-32A48D8654C2}" name="nama_tujuan" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{3D349B3F-9099-4C7B-BAAC-384CC982CC07}" name="jumlah_migran" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{A97C526F-F4CF-439B-94B7-1ACC3B0D52B8}" name="kode_asal" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{A06EB03B-EFA2-428E-8750-2625B01CC79E}" name="nama_asal" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{915F2F13-451B-4692-85C8-931B037F0D1D}" name="kode_tujuan" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{CA49676B-7235-4E1F-80E5-32A48D8654C2}" name="nama_tujuan" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{3D349B3F-9099-4C7B-BAAC-384CC982CC07}" name="jumlah_migran" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ABF51127-2134-4E4E-8D72-FB8B7593E275}" name="Table6" displayName="Table6" ref="A1:F67" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ABF51127-2134-4E4E-8D72-FB8B7593E275}" name="Table6" displayName="Table6" ref="A1:F67" totalsRowShown="0" headerRowDxfId="87" headerRowBorderDxfId="86" tableBorderDxfId="85" totalsRowBorderDxfId="84">
   <autoFilter ref="A1:F67" xr:uid="{ABF51127-2134-4E4E-8D72-FB8B7593E275}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{7E370B52-3676-4636-BA96-FA168869521E}" name="kode_asal" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{E91C0B4B-6D2C-4FF1-BF35-AF2CB7ED462D}" name="nama_asal" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{D4DEA431-DB24-4B59-8343-9560230D37B9}" name="kode_tujuan" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{3BD14680-8F12-4AE4-89DB-4D219AEAF7E6}" name="nama_tujuan" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C3139E59-C951-4BD2-AFD6-E852CF0AEBFD}" name="weight" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{DF31EAA0-1330-423A-BD93-1E09FAA67216}" name="centrality_nanti" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{7E370B52-3676-4636-BA96-FA168869521E}" name="kode_asal" dataDxfId="83"/>
+    <tableColumn id="2" xr3:uid="{E91C0B4B-6D2C-4FF1-BF35-AF2CB7ED462D}" name="nama_asal" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{D4DEA431-DB24-4B59-8343-9560230D37B9}" name="kode_tujuan" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{3BD14680-8F12-4AE4-89DB-4D219AEAF7E6}" name="nama_tujuan" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{C3139E59-C951-4BD2-AFD6-E852CF0AEBFD}" name="weight" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{DF31EAA0-1330-423A-BD93-1E09FAA67216}" name="centrality_nanti" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5833,7 +5890,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>632</v>
@@ -5859,7 +5916,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>633</v>
@@ -5885,7 +5942,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>634</v>
@@ -5911,7 +5968,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>635</v>
@@ -5937,7 +5994,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>636</v>
@@ -5963,7 +6020,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>639</v>
@@ -5989,7 +6046,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>640</v>
@@ -6015,7 +6072,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>641</v>
@@ -6033,7 +6090,7 @@
         <v>642</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>643</v>
+        <v>716</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -6041,16 +6098,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F10" s="2">
         <v>2020</v>
@@ -6059,7 +6116,7 @@
         <v>69</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -6067,10 +6124,10 @@
         <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>69</v>
@@ -6093,10 +6150,10 @@
         <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>69</v>
@@ -6119,13 +6176,13 @@
         <v>20</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>19</v>
@@ -6145,7 +6202,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>22</v>
@@ -6171,7 +6228,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>24</v>
@@ -6197,7 +6254,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>25</v>
@@ -6223,13 +6280,13 @@
         <v>20</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>19</v>
@@ -6249,7 +6306,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>27</v>
@@ -6261,10 +6318,10 @@
         <v>19</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H18" s="24" t="s">
         <v>69</v>
@@ -6275,7 +6332,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>29</v>
@@ -6290,7 +6347,7 @@
         <v>2020</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H19" s="24" t="s">
         <v>69</v>
@@ -6301,13 +6358,13 @@
         <v>20</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>19</v>
@@ -6327,16 +6384,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F21" s="2">
         <v>2020</v>
@@ -6345,7 +6402,7 @@
         <v>69</v>
       </c>
       <c r="H21" s="24" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -6353,10 +6410,10 @@
         <v>31</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>69</v>
@@ -6368,7 +6425,7 @@
         <v>2020</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H22" s="24" t="s">
         <v>69</v>
@@ -6379,10 +6436,10 @@
         <v>31</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>69</v>
@@ -6394,7 +6451,7 @@
         <v>2020</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H23" s="24" t="s">
         <v>69</v>
@@ -6405,16 +6462,16 @@
         <v>31</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F24" s="2">
         <v>2020</v>
@@ -6423,7 +6480,7 @@
         <v>69</v>
       </c>
       <c r="H24" s="24" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -6431,10 +6488,10 @@
         <v>31</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>69</v>
@@ -6446,7 +6503,7 @@
         <v>2020</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H25" s="24" t="s">
         <v>69</v>
@@ -6457,13 +6514,13 @@
         <v>31</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>19</v>
@@ -6472,7 +6529,7 @@
         <v>2020</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H26" s="24" t="s">
         <v>69</v>
@@ -6483,10 +6540,10 @@
         <v>31</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>28</v>
@@ -6495,7 +6552,7 @@
         <v>19</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>594</v>
@@ -6509,13 +6566,13 @@
         <v>31</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>19</v>
@@ -6524,7 +6581,7 @@
         <v>2020</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H28" s="24" t="s">
         <v>69</v>
@@ -6535,13 +6592,13 @@
         <v>31</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>662</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>663</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>19</v>
@@ -6561,7 +6618,7 @@
         <v>31</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>29</v>
@@ -6587,10 +6644,10 @@
         <v>31</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>637</v>
@@ -6613,16 +6670,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F32" s="2">
         <v>2020</v>
@@ -6631,7 +6688,7 @@
         <v>69</v>
       </c>
       <c r="H32" s="24" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
@@ -6639,10 +6696,10 @@
         <v>615</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>69</v>
@@ -6665,10 +6722,10 @@
         <v>615</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>69</v>
@@ -6691,10 +6748,10 @@
         <v>615</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>69</v>
@@ -6717,10 +6774,10 @@
         <v>615</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>69</v>
@@ -6743,10 +6800,10 @@
         <v>615</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>637</v>
@@ -6769,16 +6826,16 @@
         <v>615</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F38" s="2">
         <v>2019</v>
@@ -6787,18 +6844,18 @@
         <v>69</v>
       </c>
       <c r="H38" s="24" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="23" t="s">
+        <v>671</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>672</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>696</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>673</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>69</v>
@@ -6813,15 +6870,15 @@
         <v>8</v>
       </c>
       <c r="H39" s="24" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="23" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>633</v>
@@ -6839,18 +6896,18 @@
         <v>8</v>
       </c>
       <c r="H40" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="23" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>69</v>
@@ -6865,15 +6922,15 @@
         <v>8</v>
       </c>
       <c r="H41" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="23" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>635</v>
@@ -6891,18 +6948,18 @@
         <v>8</v>
       </c>
       <c r="H42" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="23" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>637</v>
@@ -6917,18 +6974,18 @@
         <v>8</v>
       </c>
       <c r="H43" s="24" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="23" t="s">
+        <v>678</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>679</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>696</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>680</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>69</v>
@@ -6943,18 +7000,18 @@
         <v>8</v>
       </c>
       <c r="H44" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="23" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>69</v>
@@ -6969,18 +7026,18 @@
         <v>8</v>
       </c>
       <c r="H45" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="23" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>69</v>
@@ -6995,18 +7052,18 @@
         <v>8</v>
       </c>
       <c r="H46" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="23" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>69</v>
@@ -7021,18 +7078,18 @@
         <v>8</v>
       </c>
       <c r="H47" s="24" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="23" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>637</v>
@@ -7047,21 +7104,21 @@
         <v>8</v>
       </c>
       <c r="H48" s="24" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="28" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="C49" s="30" t="s">
+        <v>685</v>
+      </c>
+      <c r="D49" s="30" t="s">
         <v>686</v>
-      </c>
-      <c r="D49" s="30" t="s">
-        <v>687</v>
       </c>
       <c r="E49" s="30" t="s">
         <v>19</v>
@@ -7070,7 +7127,7 @@
         <v>2020</v>
       </c>
       <c r="G49" s="30" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H49" s="31" t="s">
         <v>69</v>
@@ -7086,7 +7143,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I1157"/>
+  <dimension ref="A1:N1157"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -7101,31 +7158,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>695</v>
+      </c>
+      <c r="B1" t="s">
+        <v>694</v>
+      </c>
+      <c r="C1" t="s">
+        <v>693</v>
+      </c>
+      <c r="D1" t="s">
+        <v>692</v>
+      </c>
+      <c r="E1" t="s">
         <v>696</v>
       </c>
-      <c r="B1" t="s">
-        <v>695</v>
-      </c>
-      <c r="C1" t="s">
-        <v>694</v>
-      </c>
-      <c r="D1" t="s">
-        <v>693</v>
-      </c>
-      <c r="E1" t="s">
-        <v>697</v>
-      </c>
       <c r="F1" t="s">
+        <v>713</v>
+      </c>
+      <c r="G1" t="s">
         <v>714</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>715</v>
       </c>
-      <c r="H1" t="s">
-        <v>716</v>
-      </c>
       <c r="I1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -30905,7 +30962,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="769" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="769" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A769" s="1">
         <v>64</v>
       </c>
@@ -30936,7 +30993,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="770" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="770" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A770" s="1">
         <v>64</v>
       </c>
@@ -30967,7 +31024,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="771" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="771" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A771" s="1">
         <v>64</v>
       </c>
@@ -30998,7 +31055,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="772" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="772" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A772" s="1">
         <v>64</v>
       </c>
@@ -31029,7 +31086,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="773" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="773" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A773" s="1">
         <v>64</v>
       </c>
@@ -31060,7 +31117,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="774" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="774" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A774" s="1">
         <v>64</v>
       </c>
@@ -31091,7 +31148,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="775" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="775" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A775" s="1">
         <v>64</v>
       </c>
@@ -31122,7 +31179,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="776" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="776" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A776" s="1">
         <v>64</v>
       </c>
@@ -31153,7 +31210,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="777" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="777" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A777" s="1">
         <v>64</v>
       </c>
@@ -31184,7 +31241,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="778" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="778" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A778" s="1">
         <v>64</v>
       </c>
@@ -31215,7 +31272,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="779" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="779" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A779" s="1">
         <v>64</v>
       </c>
@@ -31246,7 +31303,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="780" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="780" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A780" s="1">
         <v>64</v>
       </c>
@@ -31277,7 +31334,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="781" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="781" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A781" s="1">
         <v>64</v>
       </c>
@@ -31308,7 +31365,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="782" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="782" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A782" s="1">
         <v>64</v>
       </c>
@@ -31339,7 +31396,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="783" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="783" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A783" s="1">
         <v>64</v>
       </c>
@@ -31370,7 +31427,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="784" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="784" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A784" s="1">
         <v>65</v>
       </c>
@@ -31383,8 +31440,8 @@
       <c r="D784" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E784" s="5">
-        <v>0</v>
+      <c r="E784" s="7">
+        <v>26</v>
       </c>
       <c r="F784" s="1" t="s">
         <v>71</v>
@@ -31400,8 +31457,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="785" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K784" s="34"/>
+      <c r="L784" s="34"/>
+      <c r="M784" s="34"/>
+      <c r="N784" s="34"/>
+    </row>
+    <row r="785" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A785" s="1">
         <v>65</v>
       </c>
@@ -31414,8 +31475,8 @@
       <c r="D785" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E785" s="5">
-        <v>0</v>
+      <c r="E785" s="7">
+        <v>320</v>
       </c>
       <c r="F785" s="1" t="s">
         <v>71</v>
@@ -31431,8 +31492,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="786" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K785" s="34"/>
+      <c r="L785" s="34"/>
+      <c r="M785" s="34"/>
+      <c r="N785" s="34"/>
+    </row>
+    <row r="786" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A786" s="1">
         <v>65</v>
       </c>
@@ -31445,8 +31510,8 @@
       <c r="D786" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E786" s="5">
-        <v>0</v>
+      <c r="E786" s="7">
+        <v>194</v>
       </c>
       <c r="F786" s="1" t="s">
         <v>71</v>
@@ -31462,8 +31527,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="787" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K786" s="34"/>
+      <c r="L786" s="34"/>
+      <c r="M786" s="34"/>
+      <c r="N786" s="34"/>
+    </row>
+    <row r="787" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A787" s="1">
         <v>65</v>
       </c>
@@ -31476,8 +31545,8 @@
       <c r="D787" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E787" s="5">
-        <v>0</v>
+      <c r="E787" s="7">
+        <v>100</v>
       </c>
       <c r="F787" s="1" t="s">
         <v>71</v>
@@ -31493,8 +31562,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="788" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K787" s="34"/>
+      <c r="L787" s="34"/>
+      <c r="M787" s="34"/>
+      <c r="N787" s="34"/>
+    </row>
+    <row r="788" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A788" s="1">
         <v>65</v>
       </c>
@@ -31507,8 +31580,8 @@
       <c r="D788" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E788" s="5">
-        <v>0</v>
+      <c r="E788" s="7">
+        <v>161</v>
       </c>
       <c r="F788" s="1" t="s">
         <v>71</v>
@@ -31524,8 +31597,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="789" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K788" s="34"/>
+      <c r="L788" s="34"/>
+      <c r="M788" s="34"/>
+      <c r="N788" s="34"/>
+    </row>
+    <row r="789" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A789" s="1">
         <v>65</v>
       </c>
@@ -31538,8 +31615,8 @@
       <c r="D789" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E789" s="5">
-        <v>0</v>
+      <c r="E789" s="7">
+        <v>92</v>
       </c>
       <c r="F789" s="1" t="s">
         <v>71</v>
@@ -31555,8 +31632,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="790" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K789" s="34"/>
+      <c r="L789" s="34"/>
+      <c r="M789" s="34"/>
+      <c r="N789" s="34"/>
+    </row>
+    <row r="790" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A790" s="1">
         <v>65</v>
       </c>
@@ -31569,8 +31650,8 @@
       <c r="D790" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E790" s="5">
-        <v>0</v>
+      <c r="E790" s="7">
+        <v>10</v>
       </c>
       <c r="F790" s="1" t="s">
         <v>71</v>
@@ -31586,8 +31667,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="791" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K790" s="34"/>
+      <c r="L790" s="34"/>
+      <c r="M790" s="34"/>
+      <c r="N790" s="34"/>
+    </row>
+    <row r="791" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A791" s="1">
         <v>65</v>
       </c>
@@ -31600,7 +31685,7 @@
       <c r="D791" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E791" s="5">
+      <c r="E791" s="7">
         <v>0</v>
       </c>
       <c r="F791" s="1" t="s">
@@ -31617,8 +31702,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="792" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K791" s="34"/>
+      <c r="L791" s="34"/>
+      <c r="M791" s="34"/>
+      <c r="N791" s="34"/>
+    </row>
+    <row r="792" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A792" s="1">
         <v>65</v>
       </c>
@@ -31631,8 +31720,8 @@
       <c r="D792" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E792" s="5">
-        <v>0</v>
+      <c r="E792" s="7">
+        <v>82</v>
       </c>
       <c r="F792" s="1" t="s">
         <v>71</v>
@@ -31648,8 +31737,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="793" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K792" s="34"/>
+      <c r="L792" s="34"/>
+      <c r="M792" s="34"/>
+      <c r="N792" s="34"/>
+    </row>
+    <row r="793" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A793" s="1">
         <v>65</v>
       </c>
@@ -31662,8 +31755,8 @@
       <c r="D793" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E793" s="5">
-        <v>0</v>
+      <c r="E793" s="7">
+        <v>73</v>
       </c>
       <c r="F793" s="1" t="s">
         <v>71</v>
@@ -31679,8 +31772,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="794" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K793" s="34"/>
+      <c r="L793" s="34"/>
+      <c r="M793" s="34"/>
+      <c r="N793" s="34"/>
+    </row>
+    <row r="794" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A794" s="1">
         <v>65</v>
       </c>
@@ -31693,8 +31790,8 @@
       <c r="D794" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E794" s="5">
-        <v>0</v>
+      <c r="E794" s="7">
+        <v>127</v>
       </c>
       <c r="F794" s="1" t="s">
         <v>71</v>
@@ -31710,8 +31807,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="795" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K794" s="34"/>
+      <c r="L794" s="34"/>
+      <c r="M794" s="34"/>
+      <c r="N794" s="34"/>
+    </row>
+    <row r="795" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A795" s="1">
         <v>65</v>
       </c>
@@ -31724,8 +31825,8 @@
       <c r="D795" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E795" s="5">
-        <v>0</v>
+      <c r="E795" s="7">
+        <v>611</v>
       </c>
       <c r="F795" s="1" t="s">
         <v>71</v>
@@ -31741,8 +31842,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="796" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K795" s="34"/>
+      <c r="L795" s="34"/>
+      <c r="M795" s="34"/>
+      <c r="N795" s="34"/>
+    </row>
+    <row r="796" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A796" s="1">
         <v>65</v>
       </c>
@@ -31755,8 +31860,8 @@
       <c r="D796" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E796" s="5">
-        <v>0</v>
+      <c r="E796" s="7">
+        <v>551</v>
       </c>
       <c r="F796" s="1" t="s">
         <v>71</v>
@@ -31772,8 +31877,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="797" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K796" s="34"/>
+      <c r="L796" s="34"/>
+      <c r="M796" s="34"/>
+      <c r="N796" s="34"/>
+    </row>
+    <row r="797" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A797" s="1">
         <v>65</v>
       </c>
@@ -31786,8 +31895,8 @@
       <c r="D797" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E797" s="5">
-        <v>0</v>
+      <c r="E797" s="7">
+        <v>587</v>
       </c>
       <c r="F797" s="1" t="s">
         <v>71</v>
@@ -31803,8 +31912,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="798" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K797" s="34"/>
+      <c r="L797" s="34"/>
+      <c r="M797" s="34"/>
+      <c r="N797" s="34"/>
+    </row>
+    <row r="798" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A798" s="1">
         <v>65</v>
       </c>
@@ -31817,8 +31930,8 @@
       <c r="D798" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E798" s="5">
-        <v>0</v>
+      <c r="E798" s="7">
+        <v>3171</v>
       </c>
       <c r="F798" s="1" t="s">
         <v>71</v>
@@ -31834,8 +31947,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="799" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K798" s="34"/>
+      <c r="L798" s="34"/>
+      <c r="M798" s="34"/>
+      <c r="N798" s="34"/>
+    </row>
+    <row r="799" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A799" s="1">
         <v>65</v>
       </c>
@@ -31848,8 +31965,8 @@
       <c r="D799" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E799" s="5">
-        <v>0</v>
+      <c r="E799" s="7">
+        <v>6</v>
       </c>
       <c r="F799" s="1" t="s">
         <v>71</v>
@@ -31865,8 +31982,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="800" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K799" s="34"/>
+      <c r="L799" s="34"/>
+      <c r="M799" s="34"/>
+      <c r="N799" s="34"/>
+    </row>
+    <row r="800" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A800" s="1">
         <v>65</v>
       </c>
@@ -31879,7 +32000,7 @@
       <c r="D800" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E800" s="5">
+      <c r="E800" s="7">
         <v>0</v>
       </c>
       <c r="F800" s="1" t="s">
@@ -31896,8 +32017,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="801" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K800" s="34"/>
+      <c r="L800" s="34"/>
+      <c r="M800" s="34"/>
+      <c r="N800" s="34"/>
+    </row>
+    <row r="801" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A801" s="1">
         <v>65</v>
       </c>
@@ -31910,8 +32035,8 @@
       <c r="D801" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E801" s="5">
-        <v>0</v>
+      <c r="E801" s="7">
+        <v>671</v>
       </c>
       <c r="F801" s="1" t="s">
         <v>71</v>
@@ -31927,8 +32052,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="802" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K801" s="34"/>
+      <c r="L801" s="34"/>
+      <c r="M801" s="34"/>
+      <c r="N801" s="34"/>
+    </row>
+    <row r="802" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A802" s="1">
         <v>65</v>
       </c>
@@ -31941,8 +32070,8 @@
       <c r="D802" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E802" s="5">
-        <v>0</v>
+      <c r="E802" s="7">
+        <v>2406</v>
       </c>
       <c r="F802" s="1" t="s">
         <v>71</v>
@@ -31958,8 +32087,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="803" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K802" s="34"/>
+      <c r="L802" s="34"/>
+      <c r="M802" s="34"/>
+      <c r="N802" s="34"/>
+    </row>
+    <row r="803" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A803" s="1">
         <v>65</v>
       </c>
@@ -31972,8 +32105,8 @@
       <c r="D803" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E803" s="5">
-        <v>0</v>
+      <c r="E803" s="7">
+        <v>66</v>
       </c>
       <c r="F803" s="1" t="s">
         <v>71</v>
@@ -31989,8 +32122,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="804" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K803" s="34"/>
+      <c r="L803" s="34"/>
+      <c r="M803" s="34"/>
+      <c r="N803" s="34"/>
+    </row>
+    <row r="804" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A804" s="1">
         <v>65</v>
       </c>
@@ -32003,8 +32140,8 @@
       <c r="D804" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E804" s="5">
-        <v>0</v>
+      <c r="E804" s="7">
+        <v>420</v>
       </c>
       <c r="F804" s="1" t="s">
         <v>71</v>
@@ -32020,8 +32157,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="805" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K804" s="34"/>
+      <c r="L804" s="34"/>
+      <c r="M804" s="34"/>
+      <c r="N804" s="34"/>
+    </row>
+    <row r="805" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A805" s="1">
         <v>65</v>
       </c>
@@ -32034,8 +32175,8 @@
       <c r="D805" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E805" s="5">
-        <v>0</v>
+      <c r="E805" s="7">
+        <v>630</v>
       </c>
       <c r="F805" s="1" t="s">
         <v>71</v>
@@ -32051,8 +32192,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="806" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K805" s="34"/>
+      <c r="L805" s="34"/>
+      <c r="M805" s="34"/>
+      <c r="N805" s="34"/>
+    </row>
+    <row r="806" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A806" s="1">
         <v>65</v>
       </c>
@@ -32065,8 +32210,8 @@
       <c r="D806" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E806" s="5">
-        <v>0</v>
+      <c r="E806" s="7">
+        <v>3994</v>
       </c>
       <c r="F806" s="1" t="s">
         <v>71</v>
@@ -32082,8 +32227,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="807" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K806" s="34"/>
+      <c r="L806" s="34"/>
+      <c r="M806" s="34"/>
+      <c r="N806" s="34"/>
+    </row>
+    <row r="807" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A807" s="1">
         <v>65</v>
       </c>
@@ -32096,8 +32245,8 @@
       <c r="D807" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E807" s="5">
-        <v>0</v>
+      <c r="E807" s="7">
+        <v>640389</v>
       </c>
       <c r="F807" s="1" t="s">
         <v>71</v>
@@ -32113,8 +32262,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="808" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K807" s="34"/>
+      <c r="L807" s="34"/>
+      <c r="M807" s="34"/>
+      <c r="N807" s="34"/>
+    </row>
+    <row r="808" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A808" s="1">
         <v>65</v>
       </c>
@@ -32127,8 +32280,8 @@
       <c r="D808" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E808" s="5">
-        <v>0</v>
+      <c r="E808" s="7">
+        <v>246</v>
       </c>
       <c r="F808" s="1" t="s">
         <v>71</v>
@@ -32144,8 +32297,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="809" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K808" s="34"/>
+      <c r="L808" s="34"/>
+      <c r="M808" s="34"/>
+      <c r="N808" s="34"/>
+    </row>
+    <row r="809" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A809" s="1">
         <v>65</v>
       </c>
@@ -32158,8 +32315,8 @@
       <c r="D809" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E809" s="5">
-        <v>0</v>
+      <c r="E809" s="7">
+        <v>2140</v>
       </c>
       <c r="F809" s="1" t="s">
         <v>71</v>
@@ -32175,8 +32332,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="810" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K809" s="34"/>
+      <c r="L809" s="34"/>
+      <c r="M809" s="34"/>
+      <c r="N809" s="34"/>
+    </row>
+    <row r="810" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A810" s="1">
         <v>65</v>
       </c>
@@ -32189,8 +32350,8 @@
       <c r="D810" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E810" s="5">
-        <v>0</v>
+      <c r="E810" s="7">
+        <v>7642</v>
       </c>
       <c r="F810" s="1" t="s">
         <v>71</v>
@@ -32206,8 +32367,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="811" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K810" s="34"/>
+      <c r="L810" s="34"/>
+      <c r="M810" s="34"/>
+      <c r="N810" s="34"/>
+    </row>
+    <row r="811" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A811" s="1">
         <v>65</v>
       </c>
@@ -32220,8 +32385,8 @@
       <c r="D811" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E811" s="5">
-        <v>0</v>
+      <c r="E811" s="7">
+        <v>635</v>
       </c>
       <c r="F811" s="1" t="s">
         <v>71</v>
@@ -32237,8 +32402,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="812" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K811" s="34"/>
+      <c r="L811" s="34"/>
+      <c r="M811" s="34"/>
+      <c r="N811" s="34"/>
+    </row>
+    <row r="812" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A812" s="1">
         <v>65</v>
       </c>
@@ -32251,8 +32420,8 @@
       <c r="D812" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E812" s="5">
-        <v>0</v>
+      <c r="E812" s="7">
+        <v>103</v>
       </c>
       <c r="F812" s="1" t="s">
         <v>71</v>
@@ -32268,8 +32437,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="813" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K812" s="34"/>
+      <c r="L812" s="34"/>
+      <c r="M812" s="34"/>
+      <c r="N812" s="34"/>
+    </row>
+    <row r="813" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A813" s="1">
         <v>65</v>
       </c>
@@ -32282,8 +32455,8 @@
       <c r="D813" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E813" s="5">
-        <v>0</v>
+      <c r="E813" s="7">
+        <v>846</v>
       </c>
       <c r="F813" s="1" t="s">
         <v>71</v>
@@ -32299,8 +32472,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="814" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K813" s="34"/>
+      <c r="L813" s="34"/>
+      <c r="M813" s="34"/>
+      <c r="N813" s="34"/>
+    </row>
+    <row r="814" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A814" s="1">
         <v>65</v>
       </c>
@@ -32313,8 +32490,8 @@
       <c r="D814" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E814" s="5">
-        <v>0</v>
+      <c r="E814" s="7">
+        <v>97</v>
       </c>
       <c r="F814" s="1" t="s">
         <v>71</v>
@@ -32330,8 +32507,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="815" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K814" s="34"/>
+      <c r="L814" s="34"/>
+      <c r="M814" s="34"/>
+      <c r="N814" s="34"/>
+    </row>
+    <row r="815" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A815" s="1">
         <v>65</v>
       </c>
@@ -32344,7 +32525,7 @@
       <c r="D815" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E815" s="5">
+      <c r="E815" s="7">
         <v>0</v>
       </c>
       <c r="F815" s="1" t="s">
@@ -32361,8 +32542,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="816" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K815" s="34"/>
+      <c r="L815" s="34"/>
+      <c r="M815" s="34"/>
+      <c r="N815" s="34"/>
+    </row>
+    <row r="816" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A816" s="1">
         <v>65</v>
       </c>
@@ -32375,8 +32560,8 @@
       <c r="D816" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E816" s="5">
-        <v>0</v>
+      <c r="E816" s="7">
+        <v>29</v>
       </c>
       <c r="F816" s="1" t="s">
         <v>71</v>
@@ -32392,8 +32577,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="817" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K816" s="34"/>
+      <c r="L816" s="34"/>
+      <c r="M816" s="34"/>
+      <c r="N816" s="34"/>
+    </row>
+    <row r="817" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A817" s="1">
         <v>65</v>
       </c>
@@ -32406,8 +32595,8 @@
       <c r="D817" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E817" s="5">
-        <v>0</v>
+      <c r="E817" s="7">
+        <v>40</v>
       </c>
       <c r="F817" s="1" t="s">
         <v>71</v>
@@ -32423,8 +32612,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="818" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K817" s="34"/>
+      <c r="L817" s="34"/>
+      <c r="M817" s="34"/>
+      <c r="N817" s="34"/>
+    </row>
+    <row r="818" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A818" s="1">
         <v>71</v>
       </c>
@@ -32454,8 +32647,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="819" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K818" s="34"/>
+      <c r="L818" s="34"/>
+      <c r="M818" s="34"/>
+      <c r="N818" s="34"/>
+    </row>
+    <row r="819" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A819" s="1">
         <v>71</v>
       </c>
@@ -32485,8 +32682,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="820" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K819" s="34"/>
+      <c r="L819" s="34"/>
+      <c r="M819" s="34"/>
+      <c r="N819" s="34"/>
+    </row>
+    <row r="820" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A820" s="1">
         <v>71</v>
       </c>
@@ -32516,8 +32717,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="821" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K820" s="34"/>
+      <c r="L820" s="34"/>
+      <c r="M820" s="34"/>
+      <c r="N820" s="34"/>
+    </row>
+    <row r="821" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A821" s="1">
         <v>71</v>
       </c>
@@ -32547,8 +32752,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="822" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K821" s="34"/>
+      <c r="L821" s="34"/>
+      <c r="M821" s="34"/>
+      <c r="N821" s="34"/>
+    </row>
+    <row r="822" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A822" s="1">
         <v>71</v>
       </c>
@@ -32578,8 +32787,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="823" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K822" s="34"/>
+      <c r="L822" s="34"/>
+      <c r="M822" s="34"/>
+      <c r="N822" s="34"/>
+    </row>
+    <row r="823" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A823" s="1">
         <v>71</v>
       </c>
@@ -32609,8 +32822,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="824" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K823" s="34"/>
+      <c r="L823" s="34"/>
+      <c r="M823" s="34"/>
+      <c r="N823" s="34"/>
+    </row>
+    <row r="824" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A824" s="1">
         <v>71</v>
       </c>
@@ -32640,8 +32857,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="825" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K824" s="34"/>
+      <c r="L824" s="34"/>
+      <c r="M824" s="34"/>
+      <c r="N824" s="34"/>
+    </row>
+    <row r="825" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A825" s="1">
         <v>71</v>
       </c>
@@ -32671,8 +32892,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="826" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K825" s="34"/>
+      <c r="L825" s="34"/>
+      <c r="M825" s="34"/>
+      <c r="N825" s="34"/>
+    </row>
+    <row r="826" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A826" s="1">
         <v>71</v>
       </c>
@@ -32702,8 +32927,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="827" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K826" s="34"/>
+      <c r="L826" s="34"/>
+      <c r="M826" s="34"/>
+      <c r="N826" s="34"/>
+    </row>
+    <row r="827" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A827" s="1">
         <v>71</v>
       </c>
@@ -32733,8 +32962,12 @@
         <f>METADATA_SOURCES!$A$2</f>
         <v>SRC001</v>
       </c>
-    </row>
-    <row r="828" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="K827" s="34"/>
+      <c r="L827" s="34"/>
+      <c r="M827" s="34"/>
+      <c r="N827" s="34"/>
+    </row>
+    <row r="828" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A828" s="1">
         <v>71</v>
       </c>
@@ -32765,7 +32998,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="829" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="829" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A829" s="1">
         <v>71</v>
       </c>
@@ -32796,7 +33029,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="830" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="830" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A830" s="1">
         <v>71</v>
       </c>
@@ -32827,7 +33060,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="831" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="831" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A831" s="1">
         <v>71</v>
       </c>
@@ -32858,7 +33091,7 @@
         <v>SRC001</v>
       </c>
     </row>
-    <row r="832" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="832" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A832" s="1">
         <v>71</v>
       </c>
@@ -42998,37 +43231,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>701</v>
+      </c>
+      <c r="B1" t="s">
         <v>702</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>704</v>
+      </c>
+      <c r="D1" t="s">
+        <v>708</v>
+      </c>
+      <c r="E1" t="s">
+        <v>709</v>
+      </c>
+      <c r="F1" t="s">
+        <v>710</v>
+      </c>
+      <c r="G1" t="s">
+        <v>711</v>
+      </c>
+      <c r="H1" t="s">
         <v>703</v>
       </c>
-      <c r="C1" t="s">
-        <v>705</v>
-      </c>
-      <c r="D1" t="s">
-        <v>709</v>
-      </c>
-      <c r="E1" t="s">
-        <v>710</v>
-      </c>
-      <c r="F1" t="s">
-        <v>711</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>706</v>
+      </c>
+      <c r="J1" t="s">
         <v>712</v>
       </c>
-      <c r="H1" t="s">
-        <v>704</v>
-      </c>
-      <c r="I1" t="s">
-        <v>707</v>
-      </c>
-      <c r="J1" t="s">
-        <v>713</v>
-      </c>
       <c r="K1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -44282,34 +44515,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>699</v>
+      </c>
+      <c r="B1" t="s">
         <v>700</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>701</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>702</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>703</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>704</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>705</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>706</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>707</v>
       </c>
-      <c r="I1" t="s">
-        <v>708</v>
-      </c>
       <c r="J1" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -61813,22 +62046,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>698</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>699</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -64839,19 +65072,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
+        <v>695</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>694</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>693</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>692</v>
+      </c>
+      <c r="E1" s="22" t="s">
         <v>696</v>
-      </c>
-      <c r="B1" s="22" t="s">
-        <v>695</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>694</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>693</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>697</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -65803,7 +66036,7 @@
         <v>42</v>
       </c>
       <c r="E57" s="8">
-        <v>0</v>
+        <v>127</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
@@ -65999,22 +66232,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="E1" s="22" t="s">
+        <v>690</v>
+      </c>
+      <c r="F1" s="20" t="s">
         <v>691</v>
-      </c>
-      <c r="F1" s="20" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -67021,7 +67254,7 @@
         <v>42</v>
       </c>
       <c r="E57" s="8">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="F57" s="15"/>
     </row>

</xml_diff>